<commit_message>
Initial commit - ScootDR project
</commit_message>
<xml_diff>
--- a/Fleet Mileage.xlsx
+++ b/Fleet Mileage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DATA/Business/scootdr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4C2B29-F795-9E45-B244-442455967A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D70E183-0643-014D-B05C-B42AEDC6D7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25540" windowHeight="15500" xr2:uid="{DD62F603-65F5-B64B-908C-44E0CEED2B19}"/>
   </bookViews>
@@ -464,9 +464,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -474,10 +471,13 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -895,57 +895,57 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C4" s="11">
-        <v>51007</v>
+        <v>53997</v>
       </c>
       <c r="D4" s="11">
-        <v>54000</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="13"/>
+        <v>57000</v>
+      </c>
       <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
+      <c r="H4" s="27" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C5" s="11">
-        <v>51002</v>
+        <v>51007</v>
       </c>
       <c r="D5" s="11">
         <v>54000</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="13"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C6" s="11">
-        <v>53997</v>
+        <v>51002</v>
       </c>
       <c r="D6" s="11">
-        <v>57000</v>
-      </c>
+        <v>54000</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="13"/>
       <c r="G6" s="26"/>
-      <c r="H6" s="27" t="s">
-        <v>50</v>
-      </c>
+      <c r="H6" s="26"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
@@ -960,8 +960,8 @@
       <c r="D7" s="11">
         <v>51000</v>
       </c>
-      <c r="G7" s="23"/>
-      <c r="H7" s="24" t="s">
+      <c r="G7" s="22"/>
+      <c r="H7" s="23" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C22" s="10">
-        <v>28960</v>
+        <v>30040</v>
       </c>
       <c r="D22" s="10">
         <v>33000</v>
@@ -1234,16 +1234,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C23" s="10">
-        <v>27101</v>
+        <v>28960</v>
       </c>
       <c r="D23" s="10">
-        <v>30000</v>
+        <v>33000</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="13"/>

</xml_diff>